<commit_message>
Visual and Step-Handover Logic Fixes
- Upgraded reactive interface with tab-locking to prevent out-of-order execution.
- Updtaed YAML-based configuration manager
- Bug fixes to submodules
</commit_message>
<xml_diff>
--- a/R/Fm_Matrices/Fm_NoPro.xlsx
+++ b/R/Fm_Matrices/Fm_NoPro.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LBQui\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LBQui\OneDrive\Desktop\Paper 1\May2026_AppMain\phytoclassShiny\R\Fm_Matrices\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EDFF3E4-D176-4161-9701-6AC57C763147}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E06B7459-84BD-4073-B18A-068C8CF60BD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Fm" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Per</t>
   </si>
@@ -59,9 +59,6 @@
   </si>
   <si>
     <t>Prasinophytes</t>
-  </si>
-  <si>
-    <t>Chlorophytes</t>
   </si>
   <si>
     <t>Cryptophytes</t>
@@ -944,7 +941,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
@@ -982,10 +979,10 @@
         <v>9</v>
       </c>
       <c r="L1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>10</v>
@@ -1055,25 +1052,25 @@
         <v>0</v>
       </c>
       <c r="E3" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="2">
         <v>0</v>
       </c>
       <c r="G3" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3" s="2">
         <v>0</v>
       </c>
       <c r="I3" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L3" s="2">
         <v>0</v>
@@ -1082,7 +1079,7 @@
         <v>0</v>
       </c>
       <c r="N3" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O3" s="2">
         <v>1</v>
@@ -1099,7 +1096,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="2">
         <v>0</v>
@@ -1114,7 +1111,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" s="2">
         <v>0</v>
@@ -1126,7 +1123,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N4" s="2">
         <v>0</v>
@@ -1140,13 +1137,13 @@
         <v>15</v>
       </c>
       <c r="B5" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C5" s="2">
         <v>0</v>
       </c>
       <c r="D5" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" s="2">
         <v>0</v>
@@ -1173,7 +1170,7 @@
         <v>0</v>
       </c>
       <c r="M5" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N5" s="2">
         <v>0</v>
@@ -1187,13 +1184,13 @@
         <v>16</v>
       </c>
       <c r="B6" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="2">
         <v>0</v>
@@ -1205,7 +1202,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" s="2">
         <v>0</v>
@@ -1220,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="M6" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N6" s="2">
         <v>0</v>
@@ -1252,7 +1249,7 @@
         <v>0</v>
       </c>
       <c r="H7" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7" s="2">
         <v>0</v>
@@ -1284,10 +1281,10 @@
         <v>0</v>
       </c>
       <c r="C8" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" s="2">
         <v>0</v>
@@ -1305,7 +1302,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8" s="2">
         <v>0</v>
@@ -1314,7 +1311,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N8" s="2">
         <v>0</v>
@@ -1334,7 +1331,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="2">
         <v>0</v>
@@ -1352,13 +1349,13 @@
         <v>0</v>
       </c>
       <c r="J9" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" s="2">
         <v>0</v>
       </c>
-      <c r="L9" s="2">
-        <v>0</v>
+      <c r="L9">
+        <v>1</v>
       </c>
       <c r="M9" s="2">
         <v>0</v>
@@ -1367,53 +1364,6 @@
         <v>0</v>
       </c>
       <c r="O9" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15">
-      <c r="A10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="1">
-        <v>0</v>
-      </c>
-      <c r="C10" s="2">
-        <v>0</v>
-      </c>
-      <c r="D10" s="2">
-        <v>1</v>
-      </c>
-      <c r="E10" s="2">
-        <v>0</v>
-      </c>
-      <c r="F10" s="2">
-        <v>0</v>
-      </c>
-      <c r="G10" s="2">
-        <v>0</v>
-      </c>
-      <c r="H10" s="2">
-        <v>0</v>
-      </c>
-      <c r="I10" s="2">
-        <v>0</v>
-      </c>
-      <c r="J10" s="2">
-        <v>0</v>
-      </c>
-      <c r="K10" s="2">
-        <v>0</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-      <c r="M10" s="2">
-        <v>0</v>
-      </c>
-      <c r="N10" s="2">
-        <v>0</v>
-      </c>
-      <c r="O10" s="2">
         <v>1</v>
       </c>
     </row>

</xml_diff>